<commit_message>
Update analysis spreadsheets with new data: revised "Omfång på lärandemål.xlsx", "Samstämmighet svenska och engelska.xlsx", and "Stavfel och språkbruk.xlsx".
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Omfång på lärandemål.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Omfång på lärandemål.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Omfång på lärandemål" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Omfång på lärandemål'!$A$1:$E$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Omfång på lärandemål'!$A$1:$E$88</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E75"/>
+  <dimension ref="A1:E88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -472,7 +472,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ABY22V</t>
+          <t>BY1054</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -482,24 +482,24 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>14 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ABY22V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1054</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ABY27W</t>
+          <t>BY1061</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -509,24 +509,24 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>12 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ABY27W</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1061</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>BY1054</t>
+          <t>GBY2MA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -541,19 +541,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>14 lärandemål (maximum rekommenderat: 12)</t>
+          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1054</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2MA</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>BY3004</t>
+          <t>GBY2NF</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -563,56 +563,56 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>9 lärandemål (maximum rekommenderat: 8 för 5 hp)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY3004</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2NF</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>GDT2JN</t>
+          <t>GBY2NG</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DTA</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>29 ord: - Praktiskt konfigurera och implementera tekniker som möjliggör trådlös kommunik…</t>
+          <t>10 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GDT2JN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2NG</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>GIK289</t>
+          <t>GBY2RN</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -622,78 +622,78 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>14 lärandemål (maximum rekommenderat: 12)</t>
+          <t>9 lärandemål (maximum rekommenderat: 8 för 5 hp)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK289</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2RN</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>GIK28T</t>
+          <t>GBY2RX</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>26 ord: - Redogöra för val av forskningsansats i relation till forskningsfrågor och kuns…</t>
+          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK28T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2RX</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>GIK2AL</t>
+          <t>GDT2JM</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>DTA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>28 ord: - manipulera (söka, lägga till, ändra och ta bort) data och skapa, ändra samt ta…</t>
+          <t>10 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2AL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GDT2JM</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>GIK2V4</t>
+          <t>GDT2JN</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>DTA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -703,127 +703,127 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>26 ord: - Analysera säkerhetsbehov inom ett hemma- eller medelstort företagsnätverk och …</t>
+          <t>29 ord: - Praktiskt konfigurera och implementera tekniker som möjliggör trådlös kommunik…</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2V4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GDT2JN</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>GIK32M</t>
+          <t>BFY226</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>FYA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>12 lärandemål (maximum rekommenderat: 10 för 10 hp)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK32M</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BFY226</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>GIK376</t>
+          <t>BFY227</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>FYA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2 lärandemål (minimum rekommenderat: 4)</t>
+          <t>9 lärandemål (maximum rekommenderat: 8 för 5 hp)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK376</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BFY227</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>GIK38G</t>
+          <t>GIE3JG</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>11 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK38G</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE3JG</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>GIK38J</t>
+          <t>GIE3JH</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK38J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE3JH</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>IK1032</t>
+          <t>AIK232</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -833,110 +833,110 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>11 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1032</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AIK232</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>GMA2ZT</t>
+          <t>GIK289</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MAA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>14 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMA2ZT</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK289</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>AMD238</t>
+          <t>GIK28T</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>17 lärandemål (maximum rekommenderat: 12)</t>
+          <t>26 ord: - Redogöra för val av forskningsansats i relation till forskningsfrågor och kuns…</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD238</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK28T</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>AMD238</t>
+          <t>GIK299</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>28 ord: - med utgångspunkt i tidigare forskning identifiera ett väl avgränsat matematikd…</t>
+          <t>11 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD238</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK299</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>AMD238</t>
+          <t>GIK2AL</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -946,78 +946,78 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>26 ord: - sammanfatta det matematikdidaktiska forskningsläget inom det valda problemområ…</t>
+          <t>28 ord: - manipulera (söka, lägga till, ändra och ta bort) data och skapa, ändra samt ta…</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD238</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2AL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>AMD238</t>
+          <t>GIK2FB</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>29 ord: - med utgångspunkt i resultaten från den systematiska litteraturstudien i delkur…</t>
+          <t>11 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD238</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2FB</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>AMD238</t>
+          <t>GIK2JX</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>29 ord: - visa fördjupad förmåga att självständigt och med relevant teorianvändning anal…</t>
+          <t>12 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD238</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2JX</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>AMD239</t>
+          <t>GIK2KM</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1027,51 +1027,51 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>17 lärandemål (maximum rekommenderat: 12)</t>
+          <t>10 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD239</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2KM</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>AMD239</t>
+          <t>GIK2PB</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>28 ord: - med utgångspunkt i tidigare forskning identifiera ett väl avgränsat  matematik…</t>
+          <t>11 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD239</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PB</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>AMD239</t>
+          <t>GIK2V4</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1081,105 +1081,105 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>28 ord: - sammanfatta det matematikdidaktiska forskningsläget inom det valda  problemomr…</t>
+          <t>26 ord: - Analysera säkerhetsbehov inom ett hemma- eller medelstort företagsnätverk och …</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD239</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2V4</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>AMD239</t>
+          <t>GIK2XZ</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>29 ord: - med utgångspunkt i resultaten från den systematiska litteraturstudien i delkur…</t>
+          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD239</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2XZ</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>AMD239</t>
+          <t>GIK34Y</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>28 ord: - visa förmåga att självständigt och med relevant teorianvändning analysera och …</t>
+          <t>10 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD239</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK34Y</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>GMD2AR</t>
+          <t>GIK376</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>För få mål</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>28 lärandemål (maximum rekommenderat: 12)</t>
+          <t>2 lärandemål (minimum rekommenderat: 3 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2AR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK376</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>GMD2GF</t>
+          <t>GIK3BY</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1189,51 +1189,51 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>24 lärandemål (maximum rekommenderat: 12)</t>
+          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK3BY</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>GMD2GF</t>
+          <t>IK1032</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För få mål</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>26 ord: - med grund i aktuella styrdokument, forskning och beprövad erfarenhet redogöra …</t>
+          <t>3 lärandemål (minimum rekommenderat: 4 för 15 hp)</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1032</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>GMD2GG</t>
+          <t>IK1064</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1243,51 +1243,51 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>24 lärandemål (maximum rekommenderat: 12)</t>
+          <t>12 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GG</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1064</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>GMD2GG</t>
+          <t>IK1066</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>26 ord: - med grund i aktuella styrdokument, forskning och beprövad erfarenhet redogöra …</t>
+          <t>11 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GG</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1066</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>GMD2TV</t>
+          <t>GMA2EY</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MAA</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1297,24 +1297,24 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>32 lärandemål (maximum rekommenderat: 12)</t>
+          <t>11 lärandemål (maximum rekommenderat: 8 för 5 hp)</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2TV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMA2EY</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>GMD2XQ</t>
+          <t>MA1042</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MAA</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1324,19 +1324,19 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>77 lärandemål (maximum rekommenderat: 12)</t>
+          <t>10 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2XQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA1042</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>GMD2XQ</t>
+          <t>AMD238</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1346,24 +1346,24 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>38 ord: - beskriva, analysera, diskutera samt tillämpa differentialekvationer av första …</t>
+          <t>17 lärandemål (maximum rekommenderat: 12 för 30 hp)</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2XQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD238</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>GMD33X</t>
+          <t>AMD238</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1373,24 +1373,24 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>45 lärandemål (maximum rekommenderat: 12)</t>
+          <t>28 ord: - med utgångspunkt i tidigare forskning identifiera ett väl avgränsat matematikd…</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33X</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD238</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>GMD33Y</t>
+          <t>AMD238</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1400,24 +1400,24 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>77 lärandemål (maximum rekommenderat: 12)</t>
+          <t>26 ord: - sammanfatta det matematikdidaktiska forskningsläget inom det valda problemområ…</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD238</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>GMD33Y</t>
+          <t>AMD238</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1432,19 +1432,19 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>37 ord: - beskriva, analysera, diskutera samt tillämpa differentialekvationer av första …</t>
+          <t>29 ord: - med utgångspunkt i resultaten från den systematiska litteraturstudien i delkur…</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD238</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>MD2022</t>
+          <t>AMD238</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1454,24 +1454,24 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>För många mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>17 lärandemål (maximum rekommenderat: 12)</t>
+          <t>29 ord: - visa fördjupad förmåga att självständigt och med relevant teorianvändning anal…</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2022</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD238</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>MD2022</t>
+          <t>AMD239</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1481,24 +1481,24 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>37 ord: - beskriva, analysera, diskutera och tillämpa differentialekvationer av första o…</t>
+          <t>17 lärandemål (maximum rekommenderat: 12 för 30 hp)</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2022</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD239</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>MD2023</t>
+          <t>AMD239</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1508,24 +1508,24 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2 lärandemål (minimum rekommenderat: 4)</t>
+          <t>28 ord: - med utgångspunkt i tidigare forskning identifiera ett väl avgränsat  matematik…</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2023</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD239</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>MD2024</t>
+          <t>AMD239</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1535,56 +1535,56 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>28 ord: - sammanfatta det matematikdidaktiska forskningsläget inom det valda  problemomr…</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2024</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD239</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>GMT338</t>
+          <t>AMD239</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>29 ord: - med utgångspunkt i resultaten från den systematiska litteraturstudien i delkur…</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT338</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD239</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>GMT343</t>
+          <t>AMD239</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1594,78 +1594,78 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>32 ord: - redogöra för centrala begrepp inom området produktionsteknik omfattande område…</t>
+          <t>28 ord: - visa förmåga att självständigt och med relevant teorianvändning analysera och …</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT343</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD239</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>GMT34R</t>
+          <t>GMD2AR</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>31 ord: - kritiskt diskutera och reflektera över hur olika typer av materialfel kan påve…</t>
+          <t>28 lärandemål (maximum rekommenderat: 12 för 30 hp)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT34R</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2AR</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>GMT3BW</t>
+          <t>GMD2GF</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>29 ord: - redogöra för innebörden av begrepp och teoretiska grunder inom statiska- och d…</t>
+          <t>24 lärandemål (maximum rekommenderat: 12 för 30 hp)</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3BW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GF</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>GMT3BW</t>
+          <t>GMD2GF</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1675,213 +1675,213 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>27 ord: - redogöra för innebörden av begrepp och teoretiska grunder inom energisystem, v…</t>
+          <t>26 ord: - med grund i aktuella styrdokument, forskning och beprövad erfarenhet redogöra …</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3BW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GF</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>GMT3J2</t>
+          <t>GMD2GG</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>24 lärandemål (maximum rekommenderat: 12 för 30 hp)</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3J2</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GG</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>GMT3J3</t>
+          <t>GMD2GG</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>26 ord: - med grund i aktuella styrdokument, forskning och beprövad erfarenhet redogöra …</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3J3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GG</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>GMT3JV</t>
+          <t>GMD2H2</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H2</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>MT1033</t>
+          <t>GMD2MH</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>1 lärandemål (minimum rekommenderat: 4)</t>
+          <t>10 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1033</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MH</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>MT1074</t>
+          <t>GMD2MJ</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>10 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1074</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MJ</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>MT2006</t>
+          <t>GMD2TV</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>32 lärandemål (maximum rekommenderat: 12 för 30 hp)</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT2006</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2TV</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>AEG225</t>
+          <t>GMD2XQ</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2 lärandemål (minimum rekommenderat: 4)</t>
+          <t>77 lärandemål (maximum rekommenderat: 15 för 90 hp)</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2XQ</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>AEG233</t>
+          <t>GMD2XQ</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1891,132 +1891,132 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>28 ord: - analysera och diskutera de fysiska processer som styr utbytet av olika typer a…</t>
+          <t>38 ord: - beskriva, analysera, diskutera samt tillämpa differentialekvationer av första …</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG233</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2XQ</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>AEG2AL</t>
+          <t>GMD33X</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>28 ord: - analysera och förklara de fysiska processer som styr utbytet hos olika typer a…</t>
+          <t>45 lärandemål (maximum rekommenderat: 15 för 45 hp)</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33X</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>AEG2AV</t>
+          <t>GMD33Y</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>77 lärandemål (maximum rekommenderat: 15 för 90 hp)</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33Y</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>AEG2C5</t>
+          <t>GMD33Y</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>37 ord: - beskriva, analysera, diskutera samt tillämpa differentialekvationer av första …</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2C5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33Y</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>EG3007</t>
+          <t>MD2022</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>27 ord: - analysera och diskutera de fysikaliska processer som styr utbytet av en termis…</t>
+          <t>17 lärandemål (maximum rekommenderat: 12 för 30 hp)</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3007</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2022</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>EG3009</t>
+          <t>MD2022</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2026,105 +2026,105 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>26 ord: - analysera olika metoder som kan användas för att skydda solvärmekretsen för sk…</t>
+          <t>37 ord: - beskriva, analysera, diskutera och tillämpa differentialekvationer av första o…</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2022</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>EG3014</t>
+          <t>MD2023</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För få mål</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>35 ord: - ange och självständigt analysera olika sätt att anpassa och designa byggnader …</t>
+          <t>2 lärandemål (minimum rekommenderat: 3 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3014</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2023</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>EG3014</t>
+          <t>GMT228</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>28 ord: - Självständigt använda beräkningsprogram och göra beräkningar på en byggnads vä…</t>
+          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3014</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT228</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>EG3015</t>
+          <t>GMT343</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>29 ord: - behärska den grundläggande geometrin och vanliga begrepp vad gäller beskrivnin…</t>
+          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT343</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>EG3015</t>
+          <t>GMT343</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2134,105 +2134,105 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>28 ord: - tillämpa beräkningsmodeller och olika instrument för att kunna analysera och a…</t>
+          <t>32 ord: - redogöra för centrala begrepp inom området produktionsteknik omfattande område…</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT343</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>EG3015</t>
+          <t>GMT344</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>32 ord: - illustrera och reflektera över hur människans behov av dagsljus i byggnader ha…</t>
+          <t>9 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT344</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>EG3020</t>
+          <t>GMT349</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>28 ord: - visa kunskap och förståelse inom energieffektivisering, inbegripet såväl överb…</t>
+          <t>11 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3020</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT349</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>EG3022</t>
+          <t>GMT34R</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>27 ord: - visa kunskap och förståelse inom solenergiteknik, inbegripet såväl överblick ö…</t>
+          <t>10 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3022</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT34R</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>EG4001</t>
+          <t>GMT34R</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2242,78 +2242,78 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>41 ord: - visa väsentligt fördjupade kunskaper och insikter om aktuellt forsknings- och …</t>
+          <t>31 ord: - kritiskt diskutera och reflektera över hur olika typer av materialfel kan påve…</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG4001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT34R</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>GEG26J</t>
+          <t>GMT3BW</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>29 ord: - redogöra för innebörden av begrepp och teoretiska grunder inom statiska- och d…</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG26J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3BW</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>GEG38F</t>
+          <t>GMT3BW</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>För få mål</t>
+          <t>Långt mål</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>27 ord: - redogöra för innebörden av begrepp och teoretiska grunder inom energisystem, v…</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG38F</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3BW</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>GEG3DU</t>
+          <t>MT1033</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2323,51 +2323,51 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>1 lärandemål (minimum rekommenderat: 3 för 2 hp)</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3DU</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1033</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>GSQ23J</t>
+          <t>MT1060</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Långt mål</t>
+          <t>För många mål</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>30 ord: - Beskriva och analysera den demografiska utvecklingen i Sverige samt vilken bet…</t>
+          <t>10 lärandemål (maximum rekommenderat: 8 för 7.5 hp)</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>GSQ25F</t>
+          <t>AEG225</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2377,24 +2377,24 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>3 lärandemål (minimum rekommenderat: 4)</t>
+          <t>2 lärandemål (minimum rekommenderat: 3 för 2.5 hp)</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25F</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>AMI23A</t>
+          <t>AEG233</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2404,24 +2404,24 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>38 ord: - visa förståelse för visual literacy, bestämma de grafiska elementen som använd…</t>
+          <t>28 ord: - analysera och diskutera de fysiska processer som styr utbytet av olika typer a…</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23A</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG233</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>MI4001</t>
+          <t>AEG2AL</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2431,44 +2431,395 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>34 ord: - Visa ett kritiskt förhållningssätt till modellering och analys och att kunna a…</t>
+          <t>28 ord: - analysera och förklara de fysiska processer som styr utbytet hos olika typer a…</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MI4001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AL</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
+          <t>EG3007</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Långt mål</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>27 ord: - analysera och diskutera de fysikaliska processer som styr utbytet av en termis…</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3007</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>EG3009</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Långt mål</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>26 ord: - analysera olika metoder som kan användas för att skydda solvärmekretsen för sk…</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3009</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>EG3014</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Långt mål</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>35 ord: - ange och självständigt analysera olika sätt att anpassa och designa byggnader …</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3014</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>EG3014</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Långt mål</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>28 ord: - Självständigt använda beräkningsprogram och göra beräkningar på en byggnads vä…</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3014</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>EG3015</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Långt mål</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>29 ord: - behärska den grundläggande geometrin och vanliga begrepp vad gäller beskrivnin…</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>EG3015</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Långt mål</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>28 ord: - tillämpa beräkningsmodeller och olika instrument för att kunna analysera och a…</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>EG3015</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Långt mål</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>32 ord: - illustrera och reflektera över hur människans behov av dagsljus i byggnader ha…</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>EG3020</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Långt mål</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>28 ord: - visa kunskap och förståelse inom energieffektivisering, inbegripet såväl överb…</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3020</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>EG3022</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Långt mål</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>27 ord: - visa kunskap och förståelse inom solenergiteknik, inbegripet såväl överblick ö…</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3022</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>EG4001</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Långt mål</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>41 ord: - visa väsentligt fördjupade kunskaper och insikter om aktuellt forsknings- och …</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG4001</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>GSQ23J</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Långt mål</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>30 ord: - Beskriva och analysera den demografiska utvecklingen i Sverige samt vilken bet…</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23J</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>AMI23A</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Långt mål</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>38 ord: - visa förståelse för visual literacy, bestämma de grafiska elementen som använd…</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23A</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>MI4001</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Långt mål</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>34 ord: - Visa ett kritiskt förhållningssätt till modellering och analys och att kunna a…</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MI4001</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
           <t>MI4002</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B88" t="inlineStr">
         <is>
           <t>XYZ</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>Långt mål</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Långt mål</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
         <is>
           <t>34 ord: - Visa ett kritiskt förhållningssätt till modellering och analys och att kunna a…</t>
         </is>
       </c>
-      <c r="E75" s="2" t="inlineStr">
+      <c r="E88" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MI4002</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E75"/>
+  <autoFilter ref="A1:E88"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -2618,6 +2969,32 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="rId146"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A75" r:id="rId147"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A76" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A77" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A78" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A79" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A80" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A81" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A82" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A83" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A84" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A85" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E85" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A86" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A87" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A88" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="rId174"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>